<commit_message>
docs: reorganizar formato de la hoja de normalización
Se reorganizó la hoja de normalización en el archivo de Excel, acomodando las tablas de izquierda a derecha para presentarlas como una única tabla continua, mejorando la organización y la legibilidad del proceso de normalización.
</commit_message>
<xml_diff>
--- a/Tercer Trimestre/Base de Datos/Normalización.xlsx
+++ b/Tercer Trimestre/Base de Datos/Normalización.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\Brandon\SENA\Panify\Tercer Trimestre\Base de Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7CE3A86-4F38-4CE2-9C6F-F4260BD91BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9186AC3-83E1-4ABB-9365-137777BBC795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10590" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -812,7 +812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -891,9 +891,6 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -958,6 +955,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="22" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1189,37 +1196,37 @@
     <col min="9" max="26" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="30"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="64"/>
+      <c r="G1" s="64"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="33"/>
+      <c r="A2" s="65"/>
+      <c r="B2" s="65"/>
+      <c r="C2" s="65"/>
+      <c r="D2" s="65"/>
+      <c r="E2" s="65"/>
+      <c r="F2" s="65"/>
+      <c r="G2" s="65"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="63"/>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -2414,7 +2421,7 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M2"/>
+    <mergeCell ref="A1:G2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2448,92 +2455,92 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="29"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="42"/>
-      <c r="B2" s="43"/>
-      <c r="C2" s="43"/>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
-      <c r="N2" s="43"/>
-      <c r="O2" s="43"/>
-      <c r="P2" s="43"/>
-      <c r="Q2" s="43"/>
-      <c r="R2" s="44"/>
+      <c r="A2" s="41"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="K2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="N2" s="42"/>
+      <c r="O2" s="42"/>
+      <c r="P2" s="42"/>
+      <c r="Q2" s="42"/>
+      <c r="R2" s="43"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" s="31"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="32"/>
-      <c r="D3" s="32"/>
-      <c r="E3" s="32"/>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32"/>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="32"/>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="32"/>
-      <c r="R3" s="33"/>
+      <c r="A3" s="30"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="32"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="35"/>
-      <c r="F9" s="35"/>
-      <c r="G9" s="35"/>
-      <c r="H9" s="36"/>
-      <c r="M9" s="46" t="s">
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="35"/>
+      <c r="M9" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="N9" s="36"/>
+      <c r="N9" s="35"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B10" s="37"/>
-      <c r="C10" s="38"/>
-      <c r="D10" s="38"/>
-      <c r="E10" s="38"/>
-      <c r="F10" s="38"/>
-      <c r="G10" s="38"/>
-      <c r="H10" s="39"/>
-      <c r="M10" s="37"/>
-      <c r="N10" s="39"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="38"/>
+      <c r="M10" s="36"/>
+      <c r="N10" s="38"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" s="9" t="s">
@@ -2710,34 +2717,34 @@
       </c>
     </row>
     <row r="20" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B20" s="47" t="s">
+      <c r="B20" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="35"/>
-      <c r="D20" s="36"/>
-      <c r="I20" s="48" t="s">
+      <c r="C20" s="34"/>
+      <c r="D20" s="35"/>
+      <c r="I20" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="J20" s="36"/>
-      <c r="N20" s="49" t="s">
+      <c r="J20" s="35"/>
+      <c r="N20" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="O20" s="35"/>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="36"/>
+      <c r="O20" s="34"/>
+      <c r="P20" s="34"/>
+      <c r="Q20" s="34"/>
+      <c r="R20" s="35"/>
     </row>
     <row r="21" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="37"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="39"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="39"/>
-      <c r="N21" s="37"/>
-      <c r="O21" s="38"/>
-      <c r="P21" s="38"/>
-      <c r="Q21" s="38"/>
-      <c r="R21" s="39"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="38"/>
+      <c r="I21" s="36"/>
+      <c r="J21" s="38"/>
+      <c r="N21" s="36"/>
+      <c r="O21" s="37"/>
+      <c r="P21" s="37"/>
+      <c r="Q21" s="37"/>
+      <c r="R21" s="38"/>
     </row>
     <row r="22" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="9" t="s">
@@ -2767,10 +2774,10 @@
       <c r="P22" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="Q22" s="50" t="s">
+      <c r="Q22" s="49" t="s">
         <v>30</v>
       </c>
-      <c r="R22" s="51"/>
+      <c r="R22" s="50"/>
     </row>
     <row r="23" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="7">
@@ -2800,10 +2807,10 @@
       <c r="P23" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="Q23" s="52" t="s">
+      <c r="Q23" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="R23" s="51"/>
+      <c r="R23" s="50"/>
     </row>
     <row r="24" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="9">
@@ -2833,10 +2840,10 @@
       <c r="P24" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="Q24" s="50" t="s">
+      <c r="Q24" s="49" t="s">
         <v>84</v>
       </c>
-      <c r="R24" s="51"/>
+      <c r="R24" s="50"/>
     </row>
     <row r="25" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="7">
@@ -2866,10 +2873,10 @@
       <c r="P25" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="Q25" s="52" t="s">
+      <c r="Q25" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="R25" s="51"/>
+      <c r="R25" s="50"/>
     </row>
     <row r="26" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="9">
@@ -2899,10 +2906,10 @@
       <c r="P26" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="Q26" s="50" t="s">
+      <c r="Q26" s="49" t="s">
         <v>91</v>
       </c>
-      <c r="R26" s="51"/>
+      <c r="R26" s="50"/>
     </row>
     <row r="27" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="7">
@@ -2932,10 +2939,10 @@
       <c r="P27" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="Q27" s="52" t="s">
+      <c r="Q27" s="51" t="s">
         <v>84</v>
       </c>
-      <c r="R27" s="51"/>
+      <c r="R27" s="50"/>
     </row>
     <row r="28" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E28" s="17"/>
@@ -2948,28 +2955,28 @@
       <c r="G29" s="17"/>
     </row>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="34" t="s">
+      <c r="B30" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="35"/>
-      <c r="F30" s="36"/>
-      <c r="K30" s="40" t="s">
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="34"/>
+      <c r="F30" s="35"/>
+      <c r="K30" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="L30" s="35"/>
-      <c r="M30" s="36"/>
+      <c r="L30" s="34"/>
+      <c r="M30" s="35"/>
     </row>
     <row r="31" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="37"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="38"/>
-      <c r="F31" s="39"/>
-      <c r="K31" s="37"/>
-      <c r="L31" s="38"/>
-      <c r="M31" s="39"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="37"/>
+      <c r="F31" s="38"/>
+      <c r="K31" s="36"/>
+      <c r="L31" s="37"/>
+      <c r="M31" s="38"/>
     </row>
     <row r="32" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="9" t="s">
@@ -4135,70 +4142,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="53" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="29"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="33"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="32"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="35"/>
-      <c r="C4" s="35"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="35"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="36"/>
-      <c r="J4" s="47" t="s">
+      <c r="B4" s="34"/>
+      <c r="C4" s="34"/>
+      <c r="D4" s="34"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="34"/>
+      <c r="G4" s="35"/>
+      <c r="J4" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="35"/>
-      <c r="L4" s="35"/>
-      <c r="M4" s="35"/>
-      <c r="N4" s="36"/>
+      <c r="K4" s="34"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="34"/>
+      <c r="N4" s="35"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A5" s="37"/>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="39"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="39"/>
+      <c r="A5" s="36"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="38"/>
+      <c r="J5" s="36"/>
+      <c r="K5" s="37"/>
+      <c r="L5" s="37"/>
+      <c r="M5" s="37"/>
+      <c r="N5" s="38"/>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -4228,11 +4235,11 @@
       <c r="K6" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="55" t="s">
+      <c r="L6" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="M6" s="56"/>
-      <c r="N6" s="51"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="50"/>
     </row>
     <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="14">
@@ -4262,11 +4269,11 @@
       <c r="K7" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="L7" s="57" t="s">
+      <c r="L7" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="M7" s="56"/>
-      <c r="N7" s="51"/>
+      <c r="M7" s="55"/>
+      <c r="N7" s="50"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
@@ -4296,11 +4303,11 @@
       <c r="K8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="L8" s="55" t="s">
+      <c r="L8" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="M8" s="56"/>
-      <c r="N8" s="51"/>
+      <c r="M8" s="55"/>
+      <c r="N8" s="50"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="14">
@@ -4330,11 +4337,11 @@
       <c r="K9" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="L9" s="57" t="s">
+      <c r="L9" s="56" t="s">
         <v>85</v>
       </c>
-      <c r="M9" s="56"/>
-      <c r="N9" s="51"/>
+      <c r="M9" s="55"/>
+      <c r="N9" s="50"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
@@ -4364,11 +4371,11 @@
       <c r="K10" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="L10" s="55" t="s">
+      <c r="L10" s="54" t="s">
         <v>88</v>
       </c>
-      <c r="M10" s="56"/>
-      <c r="N10" s="51"/>
+      <c r="M10" s="55"/>
+      <c r="N10" s="50"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="14">
@@ -4398,37 +4405,37 @@
       <c r="K11" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="L11" s="57" t="s">
+      <c r="L11" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="M11" s="56"/>
-      <c r="N11" s="51"/>
+      <c r="M11" s="55"/>
+      <c r="N11" s="50"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B15" s="48" t="s">
+      <c r="B15" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="36"/>
-      <c r="E15" s="58" t="s">
+      <c r="C15" s="35"/>
+      <c r="E15" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="F15" s="36"/>
-      <c r="K15" s="49" t="s">
+      <c r="F15" s="35"/>
+      <c r="K15" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="L15" s="35"/>
-      <c r="M15" s="35"/>
-      <c r="N15" s="36"/>
+      <c r="L15" s="34"/>
+      <c r="M15" s="34"/>
+      <c r="N15" s="35"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="37"/>
-      <c r="C16" s="39"/>
-      <c r="E16" s="37"/>
-      <c r="F16" s="39"/>
-      <c r="K16" s="37"/>
-      <c r="L16" s="38"/>
-      <c r="M16" s="38"/>
-      <c r="N16" s="39"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="38"/>
+      <c r="E16" s="36"/>
+      <c r="F16" s="38"/>
+      <c r="K16" s="36"/>
+      <c r="L16" s="37"/>
+      <c r="M16" s="37"/>
+      <c r="N16" s="38"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B17" s="9" t="s">
@@ -4594,36 +4601,36 @@
     <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="34" t="s">
+      <c r="A30" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="35"/>
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36"/>
-      <c r="H30" s="40" t="s">
+      <c r="B30" s="34"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="35"/>
+      <c r="H30" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="I30" s="35"/>
-      <c r="J30" s="36"/>
-      <c r="L30" s="53" t="s">
+      <c r="I30" s="34"/>
+      <c r="J30" s="35"/>
+      <c r="L30" s="52" t="s">
         <v>106</v>
       </c>
-      <c r="M30" s="35"/>
-      <c r="N30" s="36"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="35"/>
     </row>
     <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="37"/>
-      <c r="B31" s="38"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="38"/>
-      <c r="E31" s="39"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="38"/>
-      <c r="J31" s="39"/>
-      <c r="L31" s="37"/>
-      <c r="M31" s="38"/>
-      <c r="N31" s="39"/>
+      <c r="A31" s="36"/>
+      <c r="B31" s="37"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="37"/>
+      <c r="E31" s="38"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="38"/>
+      <c r="L31" s="36"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="38"/>
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="24" t="s">
@@ -5848,74 +5855,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1" s="59" t="s">
+      <c r="A1" s="58" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="29"/>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
-      <c r="R1" s="30"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+      <c r="J1" s="28"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
+      <c r="N1" s="28"/>
+      <c r="O1" s="28"/>
+      <c r="P1" s="28"/>
+      <c r="Q1" s="28"/>
+      <c r="R1" s="29"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="31"/>
-      <c r="B2" s="32"/>
-      <c r="C2" s="32"/>
-      <c r="D2" s="32"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="32"/>
-      <c r="I2" s="32"/>
-      <c r="J2" s="32"/>
-      <c r="K2" s="32"/>
-      <c r="L2" s="32"/>
-      <c r="M2" s="32"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="32"/>
-      <c r="P2" s="32"/>
-      <c r="Q2" s="32"/>
-      <c r="R2" s="33"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
+      <c r="O2" s="31"/>
+      <c r="P2" s="31"/>
+      <c r="Q2" s="31"/>
+      <c r="R2" s="32"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" s="35"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="35"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="36"/>
-      <c r="J5" s="60" t="s">
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="35"/>
+      <c r="J5" s="59" t="s">
         <v>35</v>
       </c>
-      <c r="K5" s="35"/>
-      <c r="L5" s="36"/>
+      <c r="K5" s="34"/>
+      <c r="L5" s="35"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="37"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="38"/>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="39"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="38"/>
-      <c r="L6" s="39"/>
+      <c r="A6" s="36"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="37"/>
+      <c r="E6" s="37"/>
+      <c r="F6" s="37"/>
+      <c r="G6" s="38"/>
+      <c r="J6" s="36"/>
+      <c r="K6" s="37"/>
+      <c r="L6" s="38"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
@@ -6110,40 +6117,40 @@
       </c>
     </row>
     <row r="16" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="48" t="s">
+      <c r="B16" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="36"/>
-      <c r="F16" s="58" t="s">
+      <c r="C16" s="35"/>
+      <c r="F16" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="G16" s="36"/>
-      <c r="I16" s="47" t="s">
+      <c r="G16" s="35"/>
+      <c r="I16" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="36"/>
-      <c r="O16" s="48" t="s">
+      <c r="J16" s="34"/>
+      <c r="K16" s="34"/>
+      <c r="L16" s="35"/>
+      <c r="O16" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-      <c r="R16" s="36"/>
+      <c r="P16" s="34"/>
+      <c r="Q16" s="34"/>
+      <c r="R16" s="35"/>
     </row>
     <row r="17" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="37"/>
-      <c r="C17" s="39"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="39"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="38"/>
-      <c r="K17" s="38"/>
-      <c r="L17" s="39"/>
-      <c r="O17" s="37"/>
-      <c r="P17" s="38"/>
-      <c r="Q17" s="38"/>
-      <c r="R17" s="39"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="38"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="38"/>
+      <c r="I17" s="36"/>
+      <c r="J17" s="37"/>
+      <c r="K17" s="37"/>
+      <c r="L17" s="38"/>
+      <c r="O17" s="36"/>
+      <c r="P17" s="37"/>
+      <c r="Q17" s="37"/>
+      <c r="R17" s="38"/>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B18" s="9" t="s">
@@ -6164,10 +6171,10 @@
       <c r="J18" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="K18" s="55" t="s">
+      <c r="K18" s="54" t="s">
         <v>70</v>
       </c>
-      <c r="L18" s="51"/>
+      <c r="L18" s="50"/>
       <c r="O18" s="26" t="s">
         <v>112</v>
       </c>
@@ -6200,10 +6207,10 @@
       <c r="J19" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="K19" s="57" t="s">
+      <c r="K19" s="56" t="s">
         <v>76</v>
       </c>
-      <c r="L19" s="51"/>
+      <c r="L19" s="50"/>
       <c r="O19" s="13">
         <v>1</v>
       </c>
@@ -6236,10 +6243,10 @@
       <c r="J20" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="K20" s="55" t="s">
+      <c r="K20" s="54" t="s">
         <v>82</v>
       </c>
-      <c r="L20" s="51"/>
+      <c r="L20" s="50"/>
       <c r="O20" s="9">
         <v>2</v>
       </c>
@@ -6272,10 +6279,10 @@
       <c r="J21" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="K21" s="57" t="s">
+      <c r="K21" s="56" t="s">
         <v>85</v>
       </c>
-      <c r="L21" s="51"/>
+      <c r="L21" s="50"/>
       <c r="O21" s="13">
         <v>3</v>
       </c>
@@ -6308,10 +6315,10 @@
       <c r="J22" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="K22" s="55" t="s">
+      <c r="K22" s="54" t="s">
         <v>88</v>
       </c>
-      <c r="L22" s="51"/>
+      <c r="L22" s="50"/>
       <c r="O22" s="9">
         <v>4</v>
       </c>
@@ -6344,10 +6351,10 @@
       <c r="J23" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="K23" s="57" t="s">
+      <c r="K23" s="56" t="s">
         <v>92</v>
       </c>
-      <c r="L23" s="51"/>
+      <c r="L23" s="50"/>
       <c r="O23" s="13">
         <v>5</v>
       </c>
@@ -6369,36 +6376,36 @@
     <row r="29" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M31" s="49" t="s">
+      <c r="M31" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="N31" s="35"/>
-      <c r="O31" s="35"/>
-      <c r="P31" s="35"/>
-      <c r="Q31" s="36"/>
+      <c r="N31" s="34"/>
+      <c r="O31" s="34"/>
+      <c r="P31" s="34"/>
+      <c r="Q31" s="35"/>
     </row>
     <row r="32" spans="2:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="34" t="s">
+      <c r="B32" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="36"/>
-      <c r="M32" s="37"/>
-      <c r="N32" s="38"/>
-      <c r="O32" s="38"/>
-      <c r="P32" s="38"/>
-      <c r="Q32" s="39"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="34"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="35"/>
+      <c r="M32" s="36"/>
+      <c r="N32" s="37"/>
+      <c r="O32" s="37"/>
+      <c r="P32" s="37"/>
+      <c r="Q32" s="38"/>
     </row>
     <row r="33" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="37"/>
-      <c r="C33" s="38"/>
-      <c r="D33" s="38"/>
-      <c r="E33" s="38"/>
-      <c r="F33" s="38"/>
-      <c r="G33" s="39"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="37"/>
+      <c r="D33" s="37"/>
+      <c r="E33" s="37"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
       <c r="M33" s="9" t="s">
         <v>72</v>
       </c>
@@ -6615,30 +6622,30 @@
     <row r="42" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H44" s="40" t="s">
+      <c r="H44" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="I44" s="35"/>
-      <c r="J44" s="35"/>
-      <c r="K44" s="36"/>
-      <c r="M44" s="53" t="s">
+      <c r="I44" s="34"/>
+      <c r="J44" s="34"/>
+      <c r="K44" s="35"/>
+      <c r="M44" s="52" t="s">
         <v>106</v>
       </c>
-      <c r="N44" s="35"/>
-      <c r="O44" s="35"/>
-      <c r="P44" s="35"/>
-      <c r="Q44" s="36"/>
+      <c r="N44" s="34"/>
+      <c r="O44" s="34"/>
+      <c r="P44" s="34"/>
+      <c r="Q44" s="35"/>
     </row>
     <row r="45" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H45" s="37"/>
-      <c r="I45" s="38"/>
-      <c r="J45" s="38"/>
-      <c r="K45" s="39"/>
-      <c r="M45" s="37"/>
-      <c r="N45" s="38"/>
-      <c r="O45" s="38"/>
-      <c r="P45" s="38"/>
-      <c r="Q45" s="39"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="37"/>
+      <c r="J45" s="37"/>
+      <c r="K45" s="38"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="37"/>
+      <c r="O45" s="37"/>
+      <c r="P45" s="37"/>
+      <c r="Q45" s="38"/>
     </row>
     <row r="46" spans="2:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H46" s="9" t="s">
@@ -7765,13 +7772,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:R2"/>
-    <mergeCell ref="A5:G6"/>
-    <mergeCell ref="J5:L6"/>
-    <mergeCell ref="B16:C17"/>
-    <mergeCell ref="F16:G17"/>
-    <mergeCell ref="I16:L17"/>
-    <mergeCell ref="O16:R17"/>
     <mergeCell ref="B32:G33"/>
     <mergeCell ref="K23:L23"/>
     <mergeCell ref="H44:K45"/>
@@ -7782,6 +7782,13 @@
     <mergeCell ref="K21:L21"/>
     <mergeCell ref="K22:L22"/>
     <mergeCell ref="M31:Q32"/>
+    <mergeCell ref="A1:R2"/>
+    <mergeCell ref="A5:G6"/>
+    <mergeCell ref="J5:L6"/>
+    <mergeCell ref="B16:C17"/>
+    <mergeCell ref="F16:G17"/>
+    <mergeCell ref="I16:L17"/>
+    <mergeCell ref="O16:R17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>